<commit_message>
Group B phase 2: user decisions 1/2/5, 12 Brennan STEPs -> FSM_MEAS / NWO_FS sizes
- 6900-05-04-O (keep W4, L2 = Brennan), 6805-08-06 N1 = Brennan, 6801-LL-08-08 = Brennan record
- FSM_MEAS -04..-20 from BRENNAN_FS2403 STEPs; NWO_FS -06..-20 from BRENNAN_FS6801 STEPs;
  FS6809 keeps its own -06 stud (nwo_fs SPEC key); flat-neck studs drawn at the flats radius
- 126 of 168 group B parts + 82 configurations of existing FS roots; regen 208 new, 0 lost/changed
- checks clean; OCP closed loops: FS straights 87 cfg / 1812 checks, FS forged 36 cfg / 876 checks, 0 off
- 6901-08-12 STEP measured, still blocked by elbow generator margins; 6901-10-08 decision open
- README, PROJECT_STATUS, dry-run call files g1..g4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/out/af/DesignTable_6801_SW2.xlsx
+++ b/tools/_out/groupB_20261021/out/af/DesignTable_6801_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK51"/>
+  <dimension ref="A1:BK52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10648,32 +10648,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>6801-LL-12-12-NWO-FG</t>
+          <t>6801-LL-08-08-NWO-FG</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.66</v>
+        <v>1.25</v>
       </c>
       <c r="C49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="D49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="E49" t="n">
-        <v>0.125</v>
+        <v>0.094</v>
       </c>
       <c r="F49" t="n">
-        <v>0.3895</v>
+        <v>0.2837</v>
       </c>
       <c r="G49" t="n">
-        <v>0.4715</v>
+        <v>0.3295</v>
       </c>
       <c r="H49" t="n">
-        <v>0.1299</v>
+        <v>0.0984</v>
       </c>
       <c r="I49" t="n">
-        <v>0.1851</v>
+        <v>0.1546</v>
       </c>
       <c r="J49" t="n">
         <v>60</v>
@@ -10682,142 +10682,142 @@
         <v>37</v>
       </c>
       <c r="L49" t="n">
-        <v>3.34</v>
+        <v>2.48</v>
       </c>
       <c r="M49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="N49" t="n">
-        <v>2.2</v>
+        <v>1.62</v>
       </c>
       <c r="O49" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="P49" t="n">
-        <v>0.027</v>
+        <v>0.019</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.63</v>
+        <v>0.4425</v>
       </c>
       <c r="R49" t="n">
         <v>75</v>
       </c>
       <c r="S49" t="n">
-        <v>0.73169</v>
+        <v>0.51518</v>
       </c>
       <c r="T49" t="n">
         <v>75</v>
       </c>
       <c r="U49" t="n">
-        <v>0.41</v>
+        <v>0.31</v>
       </c>
       <c r="V49" t="n">
-        <v>0.63</v>
+        <v>0.4425</v>
       </c>
       <c r="W49" t="n">
-        <v>0.722</v>
+        <v>0.505</v>
       </c>
       <c r="X49" t="n">
-        <v>0.05</v>
+        <v>0.041</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.4725</v>
+        <v>0.33</v>
       </c>
       <c r="Z49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="AA49" t="n">
-        <v>0.469</v>
+        <v>0.344</v>
       </c>
       <c r="AB49" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="AE49" t="n">
         <v>1.25</v>
       </c>
-      <c r="AC49" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="AD49" t="n">
-        <v>0.609</v>
-      </c>
-      <c r="AE49" t="n">
-        <v>1.66</v>
-      </c>
       <c r="AF49" t="n">
-        <v>0.609</v>
+        <v>0.391</v>
       </c>
       <c r="AG49" t="n">
-        <v>3.34</v>
+        <v>2.48</v>
       </c>
       <c r="AH49" t="n">
-        <v>1.0625</v>
+        <v>0.75</v>
       </c>
       <c r="AI49" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="AJ49" t="n">
-        <v>0.3895</v>
+        <v>0.2837</v>
       </c>
       <c r="AK49" t="n">
-        <v>0.04511</v>
+        <v>0.03383</v>
       </c>
       <c r="AL49" t="n">
-        <v>0.02083</v>
+        <v>0.01562</v>
       </c>
       <c r="AM49" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="AN49" t="n">
-        <v>1.0625</v>
+        <v>0.75</v>
       </c>
       <c r="AO49" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="AP49" t="n">
-        <v>0.469</v>
+        <v>0.344</v>
       </c>
       <c r="AQ49" t="n">
-        <v>0.04511</v>
+        <v>0.03383</v>
       </c>
       <c r="AR49" t="n">
-        <v>0.02083</v>
+        <v>0.01562</v>
       </c>
       <c r="AS49" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="AT49" t="n">
-        <v>1.0625</v>
+        <v>0.75</v>
       </c>
       <c r="AU49" t="n">
-        <v>0.796</v>
+        <v>0.593</v>
       </c>
       <c r="AV49" t="n">
-        <v>1.0625</v>
+        <v>0.75</v>
       </c>
       <c r="AW49" t="n">
-        <v>2.2</v>
+        <v>1.62</v>
       </c>
       <c r="AX49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="AY49" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="AZ49" t="n">
-        <v>0.30622</v>
+        <v>0.21601</v>
       </c>
       <c r="BA49" t="n">
-        <v>0.30622</v>
+        <v>0.21601</v>
       </c>
       <c r="BB49" t="n">
-        <v>0.61293</v>
+        <v>0.43251</v>
       </c>
       <c r="BC49" t="inlineStr">
         <is>
-          <t>6801-LL-12-12-NWO-FG</t>
+          <t>6801-LL-08-08-NWO-FG</t>
         </is>
       </c>
       <c r="BD49" t="inlineStr">
         <is>
-          <t>90 deg Male JIC x Adjustable Male ORB Elbow, 1 1/16-12 JIC x 1 1/16-12 (adjustable male ORB)</t>
+          <t>90 deg Male JIC x Adjustable Male ORB Elbow, 3/4-16 JIC x 3/4-16 (adjustable male ORB)</t>
         </is>
       </c>
       <c r="BE49" t="inlineStr">
@@ -10827,12 +10827,12 @@
       </c>
       <c r="BF49" t="inlineStr">
         <is>
-          <t>1 1/16-12 JIC</t>
+          <t>3/4-16 JIC</t>
         </is>
       </c>
       <c r="BG49" t="inlineStr">
         <is>
-          <t>1 1/16-12 (adjustable male ORB)</t>
+          <t>3/4-16 (adjustable male ORB)</t>
         </is>
       </c>
       <c r="BH49" t="inlineStr">
@@ -10842,49 +10842,49 @@
       </c>
       <c r="BI49" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21 group B: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-LL-12-12-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_GRVDIA 0.945 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
+          <t>[BRENNAN-CELL 2026-10-21: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] Air-Way s136 only (double-pass 21 rows); M matches verified 6801 family | ORB_I3 0.86 = Air-Way 6801 rows of the -08 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.344 = Air-Way 6801 rows of the -08 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
         </is>
       </c>
       <c r="BJ49" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-LL-12-12-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-LL-12-12-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M@DRIVE=M, M12@DRIVE=M7, C4HEX@HEX=C, Y@REF=Y, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule") | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21) | hex A/F raised from Air-Way 1.062 to 1.0625 (JIC thread major; 2603HX rule)</t>
+          <t>B(2) printed 7/8-14 with dims duplicating the 8-10 rows (an 8-8 takes 3/4-16; non-FG 8-8 prints it) - as-printed, likely scrambled row | Air-Way prints this row with the 6801-LL-08-10 values (M 1.31, M12 3.25, C4HEX 1, Y 0.94, D1 0.39, D2 0.48) -&gt; every dimension cell = the Brennan CAD record (user 2026-10-21 "use brennan"; = BRENNAN_6801-LL-08-08-NWO-FG: ORB tip 2.480, JIC leg 1.250) | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21)</t>
         </is>
       </c>
       <c r="BK49" t="inlineStr">
         <is>
-          <t>6801-LL-12-12-NWO-FG</t>
+          <t>6801-LL-08-08-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>6801-LL-16-16-NWO-FG</t>
+          <t>6801-LL-12-12-NWO-FG</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1.81</v>
+        <v>1.66</v>
       </c>
       <c r="C50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="D50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="E50" t="n">
         <v>0.125</v>
       </c>
       <c r="F50" t="n">
-        <v>0.4365</v>
+        <v>0.3895</v>
       </c>
       <c r="G50" t="n">
-        <v>0.5965</v>
+        <v>0.4715</v>
       </c>
       <c r="H50" t="n">
-        <v>0.1292</v>
+        <v>0.1299</v>
       </c>
       <c r="I50" t="n">
-        <v>0.1858</v>
+        <v>0.1851</v>
       </c>
       <c r="J50" t="n">
         <v>60</v>
@@ -10893,28 +10893,28 @@
         <v>37</v>
       </c>
       <c r="L50" t="n">
-        <v>3.72</v>
+        <v>3.34</v>
       </c>
       <c r="M50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="N50" t="n">
-        <v>2.58</v>
+        <v>2.2</v>
       </c>
       <c r="O50" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="P50" t="n">
         <v>0.027</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.755</v>
+        <v>0.63</v>
       </c>
       <c r="R50" t="n">
         <v>75</v>
       </c>
       <c r="S50" t="n">
-        <v>0.87603</v>
+        <v>0.73169</v>
       </c>
       <c r="T50" t="n">
         <v>75</v>
@@ -10923,49 +10923,49 @@
         <v>0.41</v>
       </c>
       <c r="V50" t="n">
-        <v>0.755</v>
+        <v>0.63</v>
       </c>
       <c r="W50" t="n">
-        <v>0.866</v>
+        <v>0.722</v>
       </c>
       <c r="X50" t="n">
         <v>0.05</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.5975</v>
+        <v>0.4725</v>
       </c>
       <c r="Z50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="AA50" t="n">
         <v>0.469</v>
       </c>
       <c r="AB50" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="AC50" t="n">
         <v>0.41</v>
       </c>
       <c r="AD50" t="n">
-        <v>0.844</v>
+        <v>0.609</v>
       </c>
       <c r="AE50" t="n">
-        <v>1.81</v>
+        <v>1.66</v>
       </c>
       <c r="AF50" t="n">
-        <v>0.844</v>
+        <v>0.609</v>
       </c>
       <c r="AG50" t="n">
-        <v>3.72</v>
+        <v>3.34</v>
       </c>
       <c r="AH50" t="n">
-        <v>1.3125</v>
+        <v>1.0625</v>
       </c>
       <c r="AI50" t="n">
         <v>0.08333</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.4365</v>
+        <v>0.3895</v>
       </c>
       <c r="AK50" t="n">
         <v>0.04511</v>
@@ -10977,7 +10977,7 @@
         <v>0.08333</v>
       </c>
       <c r="AN50" t="n">
-        <v>1.3125</v>
+        <v>1.0625</v>
       </c>
       <c r="AO50" t="n">
         <v>0.08333</v>
@@ -10995,40 +10995,40 @@
         <v>0.08333</v>
       </c>
       <c r="AT50" t="n">
-        <v>1.3125</v>
+        <v>1.0625</v>
       </c>
       <c r="AU50" t="n">
-        <v>0.899</v>
+        <v>0.796</v>
       </c>
       <c r="AV50" t="n">
-        <v>1.3125</v>
+        <v>1.0625</v>
       </c>
       <c r="AW50" t="n">
-        <v>2.58</v>
+        <v>2.2</v>
       </c>
       <c r="AX50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="AY50" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="AZ50" t="n">
-        <v>0.37839</v>
+        <v>0.30622</v>
       </c>
       <c r="BA50" t="n">
-        <v>0.37839</v>
+        <v>0.30622</v>
       </c>
       <c r="BB50" t="n">
-        <v>0.75727</v>
+        <v>0.61293</v>
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>6801-LL-16-16-NWO-FG</t>
+          <t>6801-LL-12-12-NWO-FG</t>
         </is>
       </c>
       <c r="BD50" t="inlineStr">
         <is>
-          <t>90 deg Male JIC x Adjustable Male ORB Elbow, 1 5/16-12 JIC x 1 5/16-12 (adjustable male ORB)</t>
+          <t>90 deg Male JIC x Adjustable Male ORB Elbow, 1 1/16-12 JIC x 1 1/16-12 (adjustable male ORB)</t>
         </is>
       </c>
       <c r="BE50" t="inlineStr">
@@ -11038,12 +11038,12 @@
       </c>
       <c r="BF50" t="inlineStr">
         <is>
-          <t>1 5/16-12 JIC</t>
+          <t>1 1/16-12 JIC</t>
         </is>
       </c>
       <c r="BG50" t="inlineStr">
         <is>
-          <t>1 5/16-12 (adjustable male ORB)</t>
+          <t>1 1/16-12 (adjustable male ORB)</t>
         </is>
       </c>
       <c r="BH50" t="inlineStr">
@@ -11053,49 +11053,49 @@
       </c>
       <c r="BI50" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21 group B: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-LL-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_GRVDIA 1.195 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-LL-12-12-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_GRVDIA 0.945 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
         </is>
       </c>
       <c r="BJ50" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-LL-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-LL-16-16-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M@DRIVE=M, M12@DRIVE=M7, C4HEX@HEX=C, Y@REF=Y, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule") | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21) | hex A/F raised from Air-Way 1.312 to 1.3125 (JIC thread major; 2603HX rule)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-LL-12-12-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-LL-12-12-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M@DRIVE=M, M12@DRIVE=M7, C4HEX@HEX=C, Y@REF=Y, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule") | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21) | hex A/F raised from Air-Way 1.062 to 1.0625 (JIC thread major; 2603HX rule)</t>
         </is>
       </c>
       <c r="BK50" t="inlineStr">
         <is>
-          <t>6801-LL-16-16-NWO-FG</t>
+          <t>6801-LL-12-12-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>6801-LL-20-20-NWO-FG</t>
+          <t>6801-LL-16-16-NWO-FG</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2.06</v>
+        <v>1.81</v>
       </c>
       <c r="C51" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="E51" t="n">
         <v>0.125</v>
       </c>
       <c r="F51" t="n">
-        <v>0.4316</v>
+        <v>0.4365</v>
       </c>
       <c r="G51" t="n">
-        <v>0.753</v>
+        <v>0.5965</v>
       </c>
       <c r="H51" t="n">
-        <v>0.1288</v>
+        <v>0.1292</v>
       </c>
       <c r="I51" t="n">
-        <v>0.2382</v>
+        <v>0.1858</v>
       </c>
       <c r="J51" t="n">
         <v>60</v>
@@ -11104,28 +11104,28 @@
         <v>37</v>
       </c>
       <c r="L51" t="n">
-        <v>4.41</v>
+        <v>3.72</v>
       </c>
       <c r="M51" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="N51" t="n">
-        <v>3.27</v>
+        <v>2.58</v>
       </c>
       <c r="O51" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="P51" t="n">
         <v>0.027</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.9425</v>
+        <v>0.755</v>
       </c>
       <c r="R51" t="n">
         <v>75</v>
       </c>
       <c r="S51" t="n">
-        <v>1.09253</v>
+        <v>0.87603</v>
       </c>
       <c r="T51" t="n">
         <v>75</v>
@@ -11134,49 +11134,49 @@
         <v>0.41</v>
       </c>
       <c r="V51" t="n">
-        <v>0.9425</v>
+        <v>0.755</v>
       </c>
       <c r="W51" t="n">
-        <v>1.0825</v>
+        <v>0.866</v>
       </c>
       <c r="X51" t="n">
         <v>0.05</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.7534999999999999</v>
+        <v>0.5975</v>
       </c>
       <c r="Z51" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="AA51" t="n">
         <v>0.469</v>
       </c>
       <c r="AB51" t="n">
-        <v>1.875</v>
+        <v>1.5</v>
       </c>
       <c r="AC51" t="n">
         <v>0.41</v>
       </c>
       <c r="AD51" t="n">
-        <v>1.078</v>
+        <v>0.844</v>
       </c>
       <c r="AE51" t="n">
-        <v>2.06</v>
+        <v>1.81</v>
       </c>
       <c r="AF51" t="n">
-        <v>1.078</v>
+        <v>0.844</v>
       </c>
       <c r="AG51" t="n">
-        <v>4.41</v>
+        <v>3.72</v>
       </c>
       <c r="AH51" t="n">
-        <v>1.625</v>
+        <v>1.3125</v>
       </c>
       <c r="AI51" t="n">
         <v>0.08333</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.4316</v>
+        <v>0.4365</v>
       </c>
       <c r="AK51" t="n">
         <v>0.04511</v>
@@ -11188,7 +11188,7 @@
         <v>0.08333</v>
       </c>
       <c r="AN51" t="n">
-        <v>1.625</v>
+        <v>1.3125</v>
       </c>
       <c r="AO51" t="n">
         <v>0.08333</v>
@@ -11206,73 +11206,284 @@
         <v>0.08333</v>
       </c>
       <c r="AT51" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="AV51" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="AW51" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="AX51" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="AY51" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="AZ51" t="n">
+        <v>0.37839</v>
+      </c>
+      <c r="BA51" t="n">
+        <v>0.37839</v>
+      </c>
+      <c r="BB51" t="n">
+        <v>0.75727</v>
+      </c>
+      <c r="BC51" t="inlineStr">
+        <is>
+          <t>6801-LL-16-16-NWO-FG</t>
+        </is>
+      </c>
+      <c r="BD51" t="inlineStr">
+        <is>
+          <t>90 deg Male JIC x Adjustable Male ORB Elbow, 1 5/16-12 JIC x 1 5/16-12 (adjustable male ORB)</t>
+        </is>
+      </c>
+      <c r="BE51" t="inlineStr">
+        <is>
+          <t>6801</t>
+        </is>
+      </c>
+      <c r="BF51" t="inlineStr">
+        <is>
+          <t>1 5/16-12 JIC</t>
+        </is>
+      </c>
+      <c r="BG51" t="inlineStr">
+        <is>
+          <t>1 5/16-12 (adjustable male ORB)</t>
+        </is>
+      </c>
+      <c r="BH51" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="BI51" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-LL-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_GRVDIA 1.195 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
+        </is>
+      </c>
+      <c r="BJ51" t="inlineStr">
+        <is>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-LL-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-LL-16-16-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M@DRIVE=M, M12@DRIVE=M7, C4HEX@HEX=C, Y@REF=Y, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule") | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21) | hex A/F raised from Air-Way 1.312 to 1.3125 (JIC thread major; 2603HX rule)</t>
+        </is>
+      </c>
+      <c r="BK51" t="inlineStr">
+        <is>
+          <t>6801-LL-16-16-NWO-FG</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>6801-LL-20-20-NWO-FG</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.4316</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.753</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.1288</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.2382</v>
+      </c>
+      <c r="J52" t="n">
+        <v>60</v>
+      </c>
+      <c r="K52" t="n">
+        <v>37</v>
+      </c>
+      <c r="L52" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="N52" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="R52" t="n">
+        <v>75</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1.09253</v>
+      </c>
+      <c r="T52" t="n">
+        <v>75</v>
+      </c>
+      <c r="U52" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="V52" t="n">
+        <v>0.9425</v>
+      </c>
+      <c r="W52" t="n">
+        <v>1.0825</v>
+      </c>
+      <c r="X52" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>0.7534999999999999</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>1.875</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AF52" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="AG52" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="AH52" t="n">
         <v>1.625</v>
       </c>
-      <c r="AU51" t="n">
+      <c r="AI52" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AJ52" t="n">
+        <v>0.4316</v>
+      </c>
+      <c r="AK52" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="AL52" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="AM52" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AN52" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="AO52" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AP52" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="AQ52" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="AR52" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="AS52" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AT52" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="AU52" t="n">
         <v>1.102</v>
       </c>
-      <c r="AV51" t="n">
+      <c r="AV52" t="n">
         <v>1.625</v>
       </c>
-      <c r="AW51" t="n">
+      <c r="AW52" t="n">
         <v>3.27</v>
       </c>
-      <c r="AX51" t="n">
+      <c r="AX52" t="n">
         <v>0.8125</v>
       </c>
-      <c r="AY51" t="n">
+      <c r="AY52" t="n">
         <v>0.8125</v>
       </c>
-      <c r="AZ51" t="n">
+      <c r="AZ52" t="n">
         <v>0.4686</v>
       </c>
-      <c r="BA51" t="n">
+      <c r="BA52" t="n">
         <v>0.4686</v>
       </c>
-      <c r="BB51" t="n">
+      <c r="BB52" t="n">
         <v>0.93769</v>
       </c>
-      <c r="BC51" t="inlineStr">
+      <c r="BC52" t="inlineStr">
         <is>
           <t>6801-LL-20-20-NWO-FG</t>
         </is>
       </c>
-      <c r="BD51" t="inlineStr">
+      <c r="BD52" t="inlineStr">
         <is>
           <t>90 deg Male JIC x Adjustable Male ORB Elbow, 1 5/8-12 JIC x 1 5/8-12 (adjustable male ORB)</t>
         </is>
       </c>
-      <c r="BE51" t="inlineStr">
+      <c r="BE52" t="inlineStr">
         <is>
           <t>6801</t>
         </is>
       </c>
-      <c r="BF51" t="inlineStr">
+      <c r="BF52" t="inlineStr">
         <is>
           <t>1 5/8-12 JIC</t>
         </is>
       </c>
-      <c r="BG51" t="inlineStr">
+      <c r="BG52" t="inlineStr">
         <is>
           <t>1 5/8-12 (adjustable male ORB)</t>
         </is>
       </c>
-      <c r="BH51" t="inlineStr">
+      <c r="BH52" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="BI51" t="inlineStr">
+      <c r="BI52" t="inlineStr">
         <is>
           <t>[BRENNAN-CAD 2026-10-21 group B: M@DRIVE, M12@DRIVE, C4HEX@HEX, Y@REF, D1@BORE, D2@BORE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-LL-20-20-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -20 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -20 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_GRVDIA 1.507 = Air-Way 6801 rows of the -20 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | FOLD: 6801-LL fold: the forged hex arm of the adjustable-ORB leg runs on to the longer ORB leg M12 minus the 6801 tip-to-body-face ORB_I3; JIC leg, body and adjustable ORB end as 6801 (Brennan 6801-08-08 / 6801-L-08-08 / 6801-LL-08-08-NWO-FG STEPs, tools/measure/prof.py: ORB body face 0.590 / 1.110 / 1.620, tip to body face 0.860 on all three; measured at -08-08 only) | MODEL: forged elbow body per the 2500HX pattern (Brennan 2500-06-06-FG STEP): one hex arm along each leg, A/F = max(Air-Way hex, JIC thread majors), flats normal to Z, 30deg double-cone corner puck about Z (radius = hex corner, height = flats); hex-end 75deg chamfers and edge fillets NOT modelled; JIC legs: MS33656J chain per dash (2403 table, VERIFIED vs Brennan); Thread feature over THDZ; adjustable ORB stud end (nut, washer, O-ring) - Brennan 6801-XX-XX-NWO-FG STEPs, one per ORB size -02..-32: from the body face (Air-Way LEG minus ORB_I3, = Brennan on every STEP) a round neck, the locknut (hex = Air-Way HEXB = Brennan, measured thickness, both faces chamfered 15deg to the face from the across-flats circle as MEASURED on all 12 STEPs - drawn as a revolved envelope cut to the hexagon, flats normal to Z; chamfer start drawn 0.005 outside the flats circle to avoid a tangent edge: ASSUMPTION, cosmetic), the backup washer (measured OD and thickness), the O-ring undercut (root = Air-Way groove dia = Brennan) and the male ORB thread (Air-Way thread length, Thread feature); locknut, washer and O-ring are one solid with the body, as on the Brennan STEPs (O-ring not drawn); the nut sits where Brennan shows it (backed off against the washer); no tip chamfer (as on the fixed ORB ends); each leg bore runs from its face to the axis crossing</t>
         </is>
       </c>
-      <c r="BJ51" t="inlineStr">
+      <c r="BJ52" t="inlineStr">
         <is>
           <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-LL-20-20-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-LL-20-20-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M@DRIVE=M, M12@DRIVE=M7, C4HEX@HEX=C, Y@REF=Y, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule") | 6801-LL row folded into the 6801 master: Brennan 6801-LL-08-08-NWO-FG STEP shows the ORB leg's forged hex arm simply running longer (Q-NEW-FOLD-6801L, user 2026-10-21)</t>
         </is>
       </c>
-      <c r="BK51" t="inlineStr">
+      <c r="BK52" t="inlineStr">
         <is>
           <t>6801-LL-20-20-NWO-FG</t>
         </is>

</xml_diff>